<commit_message>
iapp implementé dans le main.py
</commit_message>
<xml_diff>
--- a/data/output/Garches_Equipe_2_feuille.xlsx
+++ b/data/output/Garches_Equipe_2_feuille.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,16 +469,16 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>48.806034335,2.318441501</t>
+          <t>48.821912505,2.244080972</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Avenue  de  Stalingrad  /  Rue  Jean  Marin  Naudin / Rue  Jean  Marin  Naudin  /  Avenue  de  Stalingrad</t>
+          <t>Allée  de  Billa ncourt  /  Avenue   du  Bas-Meudon</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -494,16 +494,16 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>48.806034335,2.318441501</t>
+          <t>48.821912505,2.244080972</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Avenue  de  Stalingrad  /  Rue  Jean  Marin  Naudin / Rue  Jean  Marin  Naudin  /  Avenue  de  Stalingrad</t>
+          <t>Allée  de  Billa ncourt  /  Avenue   du  Bas-Meudon</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -519,19 +519,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>48.804543053,2.318723747</t>
+          <t>48.821912505,2.244080972</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Avenue  de  Stalingrad  /  Allée  des  Martyrs  Châteaubriant</t>
+          <t>Allée  de  Billa ncourt  /  Avenue   du  Bas-Meudon</t>
         </is>
       </c>
       <c r="D4" t="n">
         <v>2</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
@@ -544,19 +544,19 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>48.804543053,2.318723747</t>
+          <t>48.822095553,2.244890221</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Avenue  de  Stalingrad  /  Allée  des  Martyrs  Châteaubriant</t>
+          <t>Avenue   du  Bas-Meudon  /  Mail Alfred Boucher</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
@@ -569,19 +569,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>48.804543053,2.318723747</t>
+          <t>48.822359641,2.2460078</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Avenue  de  Stalingrad  /  Allée  des  Martyrs  Châteaubriant</t>
+          <t>Allée  des  Moulineaux  /  Avenue   du  Bas-Meudon / Avenue   du  Bas-Meudon  /  Allée  Maximilien Luce</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
@@ -594,19 +594,19 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>48.803768522,2.320300304</t>
+          <t>48.822359641,2.2460078</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Rue  Gustave  Courbet  /  Avenue  Victor  Hugo  D77a</t>
+          <t>Allée  des  Moulineaux  /  Avenue   du  Bas-Meudon / Avenue   du  Bas-Meudon  /  Allée  Maximilien Luce</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
@@ -619,19 +619,19 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>48.803768522,2.320300304</t>
+          <t>48.822359641,2.2460078</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Rue  Gustave  Courbet  /  Avenue  Victor  Hugo  D77a</t>
+          <t>Allée  des  Moulineaux  /  Avenue   du  Bas-Meudon / Avenue   du  Bas-Meudon  /  Allée  Maximilien Luce</t>
         </is>
       </c>
       <c r="D8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" t="n">
         <v>3</v>
-      </c>
-      <c r="E8" t="n">
-        <v>2</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
@@ -644,19 +644,19 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>48.803768522,2.320300304</t>
+          <t>48.82270332,2.247440148</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Rue  Gustave  Courbet  /  Avenue  Victor  Hugo  D77a</t>
+          <t>Avenue   du  Bas-Meudon  /  Allée  d'Issy</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
@@ -669,19 +669,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>48.803768522,2.320300304</t>
+          <t>48.82270332,2.247440148</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Rue  Gustave  Courbet  /  Avenue  Victor  Hugo  D77a</t>
+          <t>Avenue   du  Bas-Meudon  /  Allée  d'Issy</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
@@ -694,19 +694,19 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>48.804094776,2.320683591</t>
+          <t>48.82270332,2.247440148</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Avenue  Victor  Hugo  /  Allée  des  Martyrs  Châteaubriant</t>
+          <t>Avenue   du  Bas-Meudon  /  Allée  d'Issy</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
@@ -719,19 +719,19 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>48.804094776,2.320683591</t>
+          <t>48.82270332,2.247440148</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Avenue  Victor  Hugo  /  Allée  des  Martyrs  Châteaubriant</t>
+          <t>Avenue   du  Bas-Meudon  /  Allée  d'Issy</t>
         </is>
       </c>
       <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" t="n">
         <v>4</v>
-      </c>
-      <c r="E12" t="n">
-        <v>2</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
@@ -744,16 +744,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>48.803335166,2.319619916</t>
+          <t>48.822867966,2.248145339</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Allée  des  Martyrs  Châteaubriant  /  Avenue  Louis  Pasteur / Avenue  Louis  Pasteur  /  Avenue  Henri  Barbusse  D77a / Avenue  Victor  Hugo  D77a  /  Avenue  Louis  Pasteur / Rond-Point  des  Martyrs  de  Châteaubriant  /  Avenue  Henri  Barbusse  D77a / Rond-Point  des  Martyrs  de  Châteaubriant  /  Avenue  Louis  Pasteur / Rond-Point  des  Martyrs  de  Châteaubriant  /  Avenue  Victor  Hugo  D77a</t>
+          <t>Allée  des  Pont s  /  Avenue   du  Bas-Meudon / Avenue   du  Bas-Meudon  /  Allée  des  Pont s / Avenue   du  Bas-Meudon  /  Allée  Louis  Bonnier</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E13" t="n">
         <v>1</v>
@@ -769,16 +769,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>48.803335166,2.319619916</t>
+          <t>48.822867966,2.248145339</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Allée  des  Martyrs  Châteaubriant  /  Avenue  Louis  Pasteur / Avenue  Louis  Pasteur  /  Avenue  Henri  Barbusse  D77a / Avenue  Victor  Hugo  D77a  /  Avenue  Louis  Pasteur / Rond-Point  des  Martyrs  de  Châteaubriant  /  Avenue  Henri  Barbusse  D77a / Rond-Point  des  Martyrs  de  Châteaubriant  /  Avenue  Louis  Pasteur / Rond-Point  des  Martyrs  de  Châteaubriant  /  Avenue  Victor  Hugo  D77a</t>
+          <t>Allée  des  Pont s  /  Avenue   du  Bas-Meudon / Avenue   du  Bas-Meudon  /  Allée  des  Pont s / Avenue   du  Bas-Meudon  /  Allée  Louis  Bonnier</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E14" t="n">
         <v>2</v>
@@ -794,16 +794,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>48.803335166,2.319619916</t>
+          <t>48.822867966,2.248145339</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Allée  des  Martyrs  Châteaubriant  /  Avenue  Louis  Pasteur / Avenue  Louis  Pasteur  /  Avenue  Henri  Barbusse  D77a / Avenue  Victor  Hugo  D77a  /  Avenue  Louis  Pasteur / Rond-Point  des  Martyrs  de  Châteaubriant  /  Avenue  Henri  Barbusse  D77a / Rond-Point  des  Martyrs  de  Châteaubriant  /  Avenue  Louis  Pasteur / Rond-Point  des  Martyrs  de  Châteaubriant  /  Avenue  Victor  Hugo  D77a</t>
+          <t>Allée  des  Pont s  /  Avenue   du  Bas-Meudon / Avenue   du  Bas-Meudon  /  Allée  des  Pont s / Avenue   du  Bas-Meudon  /  Allée  Louis  Bonnier</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E15" t="n">
         <v>3</v>
@@ -819,19 +819,19 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>48.803193012,2.318915871</t>
+          <t>48.822867966,2.248145339</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Allée  des  Martyrs  Châteaubriant  /  Avenue  Henri  Barbusse  D77a</t>
+          <t>Allée  des  Pont s  /  Avenue   du  Bas-Meudon / Avenue   du  Bas-Meudon  /  Allée  des  Pont s / Avenue   du  Bas-Meudon  /  Allée  Louis  Bonnier</t>
         </is>
       </c>
       <c r="D16" t="n">
         <v>6</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
@@ -844,12 +844,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>48.802872738,2.318221289</t>
+          <t>48.823132929,2.249309179</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Avenue  Henri  Barbusse  D77A  /  Avenue  Henri  Barbusse  D77a</t>
+          <t>Avenue   du  Bas-Meudon  /  Boulevard  des  ÃŽles  D2 / Avenue  Jean  Monnet  /  Boulevard  des  ÃŽles  D2</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -869,12 +869,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>48.802872738,2.318221289</t>
+          <t>48.823132929,2.249309179</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Avenue  Henri  Barbusse  D77A  /  Avenue  Henri  Barbusse  D77a</t>
+          <t>Avenue   du  Bas-Meudon  /  Boulevard  des  ÃŽles  D2 / Avenue  Jean  Monnet  /  Boulevard  des  ÃŽles  D2</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -894,12 +894,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>48.802872738,2.318221289</t>
+          <t>48.823132929,2.249309179</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Avenue  Henri  Barbusse  D77A  /  Avenue  Henri  Barbusse  D77a</t>
+          <t>Avenue   du  Bas-Meudon  /  Boulevard  des  ÃŽles  D2 / Avenue  Jean  Monnet  /  Boulevard  des  ÃŽles  D2</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -919,12 +919,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>48.802872738,2.318221289</t>
+          <t>48.823132929,2.249309179</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Avenue  Henri  Barbusse  D77A  /  Avenue  Henri  Barbusse  D77a</t>
+          <t>Avenue   du  Bas-Meudon  /  Boulevard  des  ÃŽles  D2 / Avenue  Jean  Monnet  /  Boulevard  des  ÃŽles  D2</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -944,19 +944,19 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>48.802056022,2.318728319</t>
+          <t>48.823132929,2.249309179</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Rue  de  Verdun  /  Avenue  Louis  Pasteur  D77</t>
+          <t>Avenue   du  Bas-Meudon  /  Boulevard  des  ÃŽles  D2 / Avenue  Jean  Monnet  /  Boulevard  des  ÃŽles  D2</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
@@ -969,19 +969,19 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>48.800789452,2.318236971</t>
+          <t>48.823132929,2.249309179</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Rue  Gabriel  Cosson  /  Avenue  Louis  Pasteur  D77</t>
+          <t>Avenue   du  Bas-Meudon  /  Boulevard  des  ÃŽles  D2 / Avenue  Jean  Monnet  /  Boulevard  des  ÃŽles  D2</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
@@ -994,19 +994,19 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>48.800789452,2.318236971</t>
+          <t>48.823132929,2.249309179</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Rue  Gabriel  Cosson  /  Avenue  Louis  Pasteur  D77</t>
+          <t>Avenue   du  Bas-Meudon  /  Boulevard  des  ÃŽles  D2 / Avenue  Jean  Monnet  /  Boulevard  des  ÃŽles  D2</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
@@ -1019,16 +1019,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>48.799722682,2.317922576</t>
+          <t>48.821869748,2.250249377</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Rue  Jean  Longuet  /  Avenue  Louis  Pasteur  D77</t>
+          <t>Boulevard  des  ÃŽles  D2  /  Quai de  la  Bataille de  Stalingrad  D7 / Place  de  la  Résistance  /  Boulevard  des  ÃŽles  D2 / Quai de  la  Bataille de  Stalingrad  D7  /  Boulevard  des  ÃŽles  D2</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
         <v>1</v>
@@ -1044,16 +1044,16 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>48.799722682,2.317922576</t>
+          <t>48.821869748,2.250249377</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Rue  Jean  Longuet  /  Avenue  Louis  Pasteur  D77</t>
+          <t>Boulevard  des  ÃŽles  D2  /  Quai de  la  Bataille de  Stalingrad  D7 / Place  de  la  Résistance  /  Boulevard  des  ÃŽles  D2 / Quai de  la  Bataille de  Stalingrad  D7  /  Boulevard  des  ÃŽles  D2</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E25" t="n">
         <v>2</v>
@@ -1069,16 +1069,16 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>48.799722682,2.317922576</t>
+          <t>48.821869748,2.250249377</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Rue  Jean  Longuet  /  Avenue  Louis  Pasteur  D77</t>
+          <t>Boulevard  des  ÃŽles  D2  /  Quai de  la  Bataille de  Stalingrad  D7 / Place  de  la  Résistance  /  Boulevard  des  ÃŽles  D2 / Quai de  la  Bataille de  Stalingrad  D7  /  Boulevard  des  ÃŽles  D2</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E26" t="n">
         <v>3</v>
@@ -1094,16 +1094,16 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>48.799722682,2.317922576</t>
+          <t>48.821869748,2.250249377</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Rue  Jean  Longuet  /  Avenue  Louis  Pasteur  D77</t>
+          <t>Boulevard  des  ÃŽles  D2  /  Quai de  la  Bataille de  Stalingrad  D7 / Place  de  la  Résistance  /  Boulevard  des  ÃŽles  D2 / Quai de  la  Bataille de  Stalingrad  D7  /  Boulevard  des  ÃŽles  D2</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E27" t="n">
         <v>4</v>
@@ -1119,19 +1119,19 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>48.801212687,2.315028051</t>
+          <t>48.821869748,2.250249377</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Avenue  Henri  Barbusse  D77A  /  Voie  René  Rousseau / Rue  Gabriel  Cosson  /  Avenue  Henri  Barbusse  D77A</t>
+          <t>Boulevard  des  ÃŽles  D2  /  Quai de  la  Bataille de  Stalingrad  D7 / Place  de  la  Résistance  /  Boulevard  des  ÃŽles  D2 / Quai de  la  Bataille de  Stalingrad  D7  /  Boulevard  des  ÃŽles  D2</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
@@ -1144,19 +1144,19 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>48.801212687,2.315028051</t>
+          <t>48.821869748,2.250249377</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Avenue  Henri  Barbusse  D77A  /  Voie  René  Rousseau / Rue  Gabriel  Cosson  /  Avenue  Henri  Barbusse  D77A</t>
+          <t>Boulevard  des  ÃŽles  D2  /  Quai de  la  Bataille de  Stalingrad  D7 / Place  de  la  Résistance  /  Boulevard  des  ÃŽles  D2 / Quai de  la  Bataille de  Stalingrad  D7  /  Boulevard  des  ÃŽles  D2</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
@@ -1169,19 +1169,19 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>48.801212687,2.315028051</t>
+          <t>48.818192406,2.247366134</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Avenue  Henri  Barbusse  D77A  /  Voie  René  Rousseau / Rue  Gabriel  Cosson  /  Avenue  Henri  Barbusse  D77A</t>
+          <t>Allée  de  la  Ferme  /  Avenue  de  Verdun  D989</t>
         </is>
       </c>
       <c r="D30" t="n">
         <v>11</v>
       </c>
       <c r="E30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
@@ -1194,12 +1194,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>48.802006004,2.31651263</t>
+          <t>48.818466626,2.245882939</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Rue  de  Verdun  /  Avenue  Henri  Barbusse  D77A</t>
+          <t>Avenue  de  Verdun  D989  /  Place  Tony de  Graaff / Avenue  de  Verdun  /  Rue  de  Meudon / Avenue  de  Verdun  D989  /  Rue   du   Docteur  Vuillième / Rue  de  Meudon  /  Avenue  de  Verdun  D989 / Rue   du   Docteur  Vuillième  /  Avenue  de  Verdun  D989</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1219,12 +1219,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>48.802006004,2.31651263</t>
+          <t>48.818466626,2.245882939</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Rue  de  Verdun  /  Avenue  Henri  Barbusse  D77A</t>
+          <t>Avenue  de  Verdun  D989  /  Place  Tony de  Graaff / Avenue  de  Verdun  /  Rue  de  Meudon / Avenue  de  Verdun  D989  /  Rue   du   Docteur  Vuillième / Rue  de  Meudon  /  Avenue  de  Verdun  D989 / Rue   du   Docteur  Vuillième  /  Avenue  de  Verdun  D989</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1238,6 +1238,831 @@
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
     </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>2</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>48.818466626,2.245882939</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  D989  /  Place  Tony de  Graaff / Avenue  de  Verdun  /  Rue  de  Meudon / Avenue  de  Verdun  D989  /  Rue   du   Docteur  Vuillième / Rue  de  Meudon  /  Avenue  de  Verdun  D989 / Rue   du   Docteur  Vuillième  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>12</v>
+      </c>
+      <c r="E33" t="n">
+        <v>3</v>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>2</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>48.818466626,2.245882939</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  D989  /  Place  Tony de  Graaff / Avenue  de  Verdun  /  Rue  de  Meudon / Avenue  de  Verdun  D989  /  Rue   du   Docteur  Vuillième / Rue  de  Meudon  /  Avenue  de  Verdun  D989 / Rue   du   Docteur  Vuillième  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>12</v>
+      </c>
+      <c r="E34" t="n">
+        <v>4</v>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>2</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>48.818466626,2.245882939</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  D989  /  Place  Tony de  Graaff / Avenue  de  Verdun  /  Rue  de  Meudon / Avenue  de  Verdun  D989  /  Rue   du   Docteur  Vuillième / Rue  de  Meudon  /  Avenue  de  Verdun  D989 / Rue   du   Docteur  Vuillième  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>12</v>
+      </c>
+      <c r="E35" t="n">
+        <v>5</v>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>2</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>48.818466626,2.245882939</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  D989  /  Place  Tony de  Graaff / Avenue  de  Verdun  /  Rue  de  Meudon / Avenue  de  Verdun  D989  /  Rue   du   Docteur  Vuillième / Rue  de  Meudon  /  Avenue  de  Verdun  D989 / Rue   du   Docteur  Vuillième  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>12</v>
+      </c>
+      <c r="E36" t="n">
+        <v>6</v>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>2</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>48.818466626,2.245882939</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  D989  /  Place  Tony de  Graaff / Avenue  de  Verdun  /  Rue  de  Meudon / Avenue  de  Verdun  D989  /  Rue   du   Docteur  Vuillième / Rue  de  Meudon  /  Avenue  de  Verdun  D989 / Rue   du   Docteur  Vuillième  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>12</v>
+      </c>
+      <c r="E37" t="n">
+        <v>7</v>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>2</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>48.818466626,2.245882939</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  D989  /  Place  Tony de  Graaff / Avenue  de  Verdun  /  Rue  de  Meudon / Avenue  de  Verdun  D989  /  Rue   du   Docteur  Vuillième / Rue  de  Meudon  /  Avenue  de  Verdun  D989 / Rue   du   Docteur  Vuillième  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>12</v>
+      </c>
+      <c r="E38" t="n">
+        <v>8</v>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>2</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>48.818466626,2.245882939</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  D989  /  Place  Tony de  Graaff / Avenue  de  Verdun  /  Rue  de  Meudon / Avenue  de  Verdun  D989  /  Rue   du   Docteur  Vuillième / Rue  de  Meudon  /  Avenue  de  Verdun  D989 / Rue   du   Docteur  Vuillième  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>12</v>
+      </c>
+      <c r="E39" t="n">
+        <v>9</v>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>2</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>48.818610293,2.245169319</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  /  Rue  Gabriel  Thomas</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>13</v>
+      </c>
+      <c r="E40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>2</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>48.818610293,2.245169319</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  /  Rue  Gabriel  Thomas</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>13</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>2</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>48.818610293,2.245169319</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  /  Rue  Gabriel  Thomas</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>13</v>
+      </c>
+      <c r="E42" t="n">
+        <v>3</v>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>2</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>48.818890946,2.24370838</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Rue  Marcel  Miquel  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>14</v>
+      </c>
+      <c r="E43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>2</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>48.818890946,2.24370838</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Rue  Marcel  Miquel  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>14</v>
+      </c>
+      <c r="E44" t="n">
+        <v>2</v>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>2</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>48.818890946,2.24370838</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Rue  Marcel  Miquel  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>14</v>
+      </c>
+      <c r="E45" t="n">
+        <v>3</v>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>2</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>48.818890946,2.24370838</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Rue  Marcel  Miquel  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>14</v>
+      </c>
+      <c r="E46" t="n">
+        <v>4</v>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>2</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>48.818890946,2.24370838</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Rue  Marcel  Miquel  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>14</v>
+      </c>
+      <c r="E47" t="n">
+        <v>5</v>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>2</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>48.81930032,2.242712451</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Rue  de  Vaugirard  D989  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>15</v>
+      </c>
+      <c r="E48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>2</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>48.81930032,2.242712451</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Rue  de  Vaugirard  D989  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>15</v>
+      </c>
+      <c r="E49" t="n">
+        <v>2</v>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>2</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>48.81930032,2.242712451</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Rue  de  Vaugirard  D989  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>15</v>
+      </c>
+      <c r="E50" t="n">
+        <v>3</v>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>2</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>48.81930032,2.242712451</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Rue  de  Vaugirard  D989  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>15</v>
+      </c>
+      <c r="E51" t="n">
+        <v>4</v>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>2</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>48.817810622,2.249042519</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  D989  /  Carrefour de  la  Ferme / Avenue  de  Verdun  D989  /  Chemin de  Saint-Cloud / Avenue  de  Verdun  D989  /  Rue  de  Paris / Chemin de  Saint-Cloud  /  Avenue  de  Verdun / Rue  Jean-Pierre  Timbaud  D101  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>16</v>
+      </c>
+      <c r="E52" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>2</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>48.817810622,2.249042519</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  D989  /  Carrefour de  la  Ferme / Avenue  de  Verdun  D989  /  Chemin de  Saint-Cloud / Avenue  de  Verdun  D989  /  Rue  de  Paris / Chemin de  Saint-Cloud  /  Avenue  de  Verdun / Rue  Jean-Pierre  Timbaud  D101  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>16</v>
+      </c>
+      <c r="E53" t="n">
+        <v>2</v>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>2</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>48.817810622,2.249042519</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  D989  /  Carrefour de  la  Ferme / Avenue  de  Verdun  D989  /  Chemin de  Saint-Cloud / Avenue  de  Verdun  D989  /  Rue  de  Paris / Chemin de  Saint-Cloud  /  Avenue  de  Verdun / Rue  Jean-Pierre  Timbaud  D101  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>16</v>
+      </c>
+      <c r="E54" t="n">
+        <v>3</v>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>2</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>48.817810622,2.249042519</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  D989  /  Carrefour de  la  Ferme / Avenue  de  Verdun  D989  /  Chemin de  Saint-Cloud / Avenue  de  Verdun  D989  /  Rue  de  Paris / Chemin de  Saint-Cloud  /  Avenue  de  Verdun / Rue  Jean-Pierre  Timbaud  D101  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>16</v>
+      </c>
+      <c r="E55" t="n">
+        <v>4</v>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>2</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>48.817810622,2.249042519</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  D989  /  Carrefour de  la  Ferme / Avenue  de  Verdun  D989  /  Chemin de  Saint-Cloud / Avenue  de  Verdun  D989  /  Rue  de  Paris / Chemin de  Saint-Cloud  /  Avenue  de  Verdun / Rue  Jean-Pierre  Timbaud  D101  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>16</v>
+      </c>
+      <c r="E56" t="n">
+        <v>5</v>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>2</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>48.817810622,2.249042519</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  D989  /  Carrefour de  la  Ferme / Avenue  de  Verdun  D989  /  Chemin de  Saint-Cloud / Avenue  de  Verdun  D989  /  Rue  de  Paris / Chemin de  Saint-Cloud  /  Avenue  de  Verdun / Rue  Jean-Pierre  Timbaud  D101  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>16</v>
+      </c>
+      <c r="E57" t="n">
+        <v>6</v>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>2</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>48.817810622,2.249042519</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  D989  /  Carrefour de  la  Ferme / Avenue  de  Verdun  D989  /  Chemin de  Saint-Cloud / Avenue  de  Verdun  D989  /  Rue  de  Paris / Chemin de  Saint-Cloud  /  Avenue  de  Verdun / Rue  Jean-Pierre  Timbaud  D101  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>16</v>
+      </c>
+      <c r="E58" t="n">
+        <v>7</v>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>2</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>48.81799295,2.250857022</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Allée  de  la  Brasserie  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>17</v>
+      </c>
+      <c r="E59" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>2</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>48.818083541,2.251255985</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  D989  /  Chemin des  Montquartiers</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>18</v>
+      </c>
+      <c r="E60" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>48.818083541,2.251255985</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  D989  /  Chemin des  Montquartiers</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>18</v>
+      </c>
+      <c r="E61" t="n">
+        <v>2</v>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>48.818274966,2.251818331</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Rue   du   Docteur  Lombard  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>19</v>
+      </c>
+      <c r="E62" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>2</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>48.818274966,2.251818331</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Rue   du   Docteur  Lombard  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>19</v>
+      </c>
+      <c r="E63" t="n">
+        <v>2</v>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>2</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>48.818958475,2.254043502</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  D989  /  Cours  Saint-Vincent / Chemin des  Vignes  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>21</v>
+      </c>
+      <c r="E64" t="n">
+        <v>1</v>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>2</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>48.818958475,2.254043502</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Avenue  de  Verdun  D989  /  Cours  Saint-Vincent / Chemin des  Vignes  /  Avenue  de  Verdun  D989</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>21</v>
+      </c>
+      <c r="E65" t="n">
+        <v>2</v>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>